<commit_message>
Apply case study stress-test decisions
</commit_message>
<xml_diff>
--- a/stage-2/22_opportunity_scoring_model.xlsx
+++ b/stage-2/22_opportunity_scoring_model.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring model" sheetId="1" r:id="Rc52afe0419914326"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R6975c3fe5e3546d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision log" sheetId="3" r:id="R52602568135844e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring model" sheetId="1" r:id="R5f59600ad1a44240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="2" r:id="R5f56755daa8a4305"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision log" sheetId="3" r:id="R13c71c89985f4445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="4" r:id="Rc502a944ff5a4611"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -476,7 +477,8 @@
     <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -491,10 +493,11 @@
       <x:c r="G1" s="34"/>
       <x:c r="H1" s="34"/>
       <x:c r="I1" s="34"/>
+      <x:c r="J1" s="34"/>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
       <x:c r="A2" s="35" t="str">
-        <x:v>Amazon India | RICE plus strategic alignment and evidence strength</x:v>
+        <x:v>Amazon India | RICE plus strategic alignment, evidence strength, and sensitivity</x:v>
       </x:c>
       <x:c r="B2" s="34"/>
       <x:c r="C2" s="34"/>
@@ -504,6 +507,7 @@
       <x:c r="G2" s="34"/>
       <x:c r="H2" s="34"/>
       <x:c r="I2" s="34"/>
+      <x:c r="J2" s="34"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="34"/>
@@ -515,6 +519,7 @@
       <x:c r="G3" s="34"/>
       <x:c r="H3" s="34"/>
       <x:c r="I3" s="34"/>
+      <x:c r="J3" s="34"/>
     </x:row>
     <x:row r="4" ht="34" customHeight="1">
       <x:c r="A4" s="36" t="str">
@@ -541,13 +546,16 @@
       <x:c r="H4" s="37" t="str">
         <x:v>Evidence strength</x:v>
       </x:c>
-      <x:c r="I4" s="38" t="str">
+      <x:c r="I4" s="37" t="str">
+        <x:v>Adjusted priority</x:v>
+      </x:c>
+      <x:c r="J4" s="38" t="str">
         <x:v>Recommendation</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="42" customHeight="1">
       <x:c r="A5" s="39" t="str">
-        <x:v>Unified exception timeline + ownership</x:v>
+        <x:v>Delivered-but-not-received resolution layer</x:v>
       </x:c>
       <x:c r="B5" s="39" t="n">
         <x:v>8</x:v>
@@ -571,7 +579,11 @@
       <x:c r="H5" s="39" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="I5" s="39" t="str">
+      <x:c r="I5" s="40" t="n">
+        <x:f>F5*G5*H5/25</x:f>
+        <x:v>3.8400000000000007</x:v>
+      </x:c>
+      <x:c r="J5" s="39" t="str">
         <x:v>Primary</x:v>
       </x:c>
     </x:row>
@@ -601,8 +613,12 @@
       <x:c r="H6" s="41" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I6" s="41" t="str">
-        <x:v>Backup / vertical slice</x:v>
+      <x:c r="I6" s="42" t="n">
+        <x:f>F6*G6*H6/25</x:f>
+        <x:v>2.448</x:v>
+      </x:c>
+      <x:c r="J6" s="41" t="str">
+        <x:v>Backup / adjacent</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -631,7 +647,11 @@
       <x:c r="H7" s="41" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I7" s="41" t="str">
+      <x:c r="I7" s="42" t="n">
+        <x:f>F7*G7*H7/25</x:f>
+        <x:v>2.1504000000000003</x:v>
+      </x:c>
+      <x:c r="J7" s="41" t="str">
         <x:v>Enabler</x:v>
       </x:c>
     </x:row>
@@ -661,7 +681,11 @@
       <x:c r="H8" s="41" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="I8" s="41" t="str">
+      <x:c r="I8" s="42" t="n">
+        <x:f>F8*G8*H8/25</x:f>
+        <x:v>1.47</x:v>
+      </x:c>
+      <x:c r="J8" s="41" t="str">
         <x:v>Backup / later</x:v>
       </x:c>
     </x:row>
@@ -691,7 +715,11 @@
       <x:c r="H9" s="41" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="I9" s="41" t="str">
+      <x:c r="I9" s="42" t="n">
+        <x:f>F9*G9*H9/25</x:f>
+        <x:v>0.54</x:v>
+      </x:c>
+      <x:c r="J9" s="41" t="str">
         <x:v>Later</x:v>
       </x:c>
     </x:row>
@@ -721,7 +749,11 @@
       <x:c r="H10" s="41" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="I10" s="41" t="str">
+      <x:c r="I10" s="42" t="n">
+        <x:f>F10*G10*H10/25</x:f>
+        <x:v>0.43199999999999994</x:v>
+      </x:c>
+      <x:c r="J10" s="41" t="str">
         <x:v>Later / edge case</x:v>
       </x:c>
     </x:row>
@@ -736,7 +768,8 @@
       <x:c r="F11" s="41"/>
       <x:c r="G11" s="41"/>
       <x:c r="H11" s="41"/>
-      <x:c r="I11" s="41" t="str">
+      <x:c r="I11" s="41"/>
+      <x:c r="J11" s="41" t="str">
         <x:v>Select the highest evidence-adjusted opportunity that can be scoped to an MVP.</x:v>
       </x:c>
     </x:row>
@@ -752,12 +785,13 @@
       <x:c r="G12" s="43"/>
       <x:c r="H12" s="43"/>
       <x:c r="I12" s="43"/>
+      <x:c r="J12" s="43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:I1"/>
-    <x:mergeCell ref="A2:I2"/>
-    <x:mergeCell ref="A12:I12"/>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+    <x:mergeCell ref="A12:J12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -998,7 +1032,7 @@
         <x:v>Problem area</x:v>
       </x:c>
       <x:c r="C5" s="44" t="str">
-        <x:v>Approve unified post-purchase exception resolution</x:v>
+        <x:v>Approve bounded delivered-but-not-received resolution layer</x:v>
       </x:c>
       <x:c r="D5" s="44" t="str">
         <x:v>Awaiting approval</x:v>
@@ -1014,7 +1048,7 @@
         <x:v>MVP exception type</x:v>
       </x:c>
       <x:c r="C6" s="41" t="str">
-        <x:v>Approve delivered but not received, or select refund-pending</x:v>
+        <x:v>Approve delivered but not received as first MVP; retain refund-pending as adjacent</x:v>
       </x:c>
       <x:c r="D6" s="41" t="str">
         <x:v>Awaiting approval</x:v>
@@ -1030,7 +1064,7 @@
         <x:v>Strategic option</x:v>
       </x:c>
       <x:c r="C7" s="41" t="str">
-        <x:v>Approve Option A; use refund transparency/support ownership as slices</x:v>
+        <x:v>Approve Option A; use support ownership as an enabler and refund transparency as adjacent</x:v>
       </x:c>
       <x:c r="D7" s="41" t="str">
         <x:v>Awaiting approval</x:v>
@@ -1082,4 +1116,255 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="10" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="10" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="52" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="33" t="str">
+        <x:v>Scoring Sensitivity</x:v>
+      </x:c>
+      <x:c r="B1" s="34"/>
+      <x:c r="C1" s="34"/>
+      <x:c r="D1" s="34"/>
+      <x:c r="E1" s="34"/>
+      <x:c r="F1" s="34"/>
+      <x:c r="G1" s="34"/>
+      <x:c r="H1" s="34"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="35" t="str">
+        <x:v>Test whether the delivered-but-not-received recommendation survives reasonable assumption changes.</x:v>
+      </x:c>
+      <x:c r="B2" s="34"/>
+      <x:c r="C2" s="34"/>
+      <x:c r="D2" s="34"/>
+      <x:c r="E2" s="34"/>
+      <x:c r="F2" s="34"/>
+      <x:c r="G2" s="34"/>
+      <x:c r="H2" s="34"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="34"/>
+      <x:c r="B3" s="34"/>
+      <x:c r="C3" s="34"/>
+      <x:c r="D3" s="34"/>
+      <x:c r="E3" s="34"/>
+      <x:c r="F3" s="34"/>
+      <x:c r="G3" s="34"/>
+      <x:c r="H3" s="34"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="36" t="str">
+        <x:v>Scenario</x:v>
+      </x:c>
+      <x:c r="B4" s="37" t="str">
+        <x:v>Reach</x:v>
+      </x:c>
+      <x:c r="C4" s="37" t="str">
+        <x:v>Impact</x:v>
+      </x:c>
+      <x:c r="D4" s="37" t="str">
+        <x:v>Confidence</x:v>
+      </x:c>
+      <x:c r="E4" s="37" t="str">
+        <x:v>Effort</x:v>
+      </x:c>
+      <x:c r="F4" s="37" t="str">
+        <x:v>RICE</x:v>
+      </x:c>
+      <x:c r="G4" s="37" t="str">
+        <x:v>Adjusted priority</x:v>
+      </x:c>
+      <x:c r="H4" s="38" t="str">
+        <x:v>Interpretation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="42" customHeight="1">
+      <x:c r="A5" s="39" t="str">
+        <x:v>Base case</x:v>
+      </x:c>
+      <x:c r="B5" s="39" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C5" s="39" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D5" s="40" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="E5" s="39" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F5" s="40" t="n">
+        <x:f>B5*C5*D5/E5</x:f>
+        <x:v>3.8400000000000007</x:v>
+      </x:c>
+      <x:c r="G5" s="40" t="n">
+        <x:f>F5*5*5/25</x:f>
+        <x:v>3.8400000000000007</x:v>
+      </x:c>
+      <x:c r="H5" s="39" t="str">
+        <x:v>Primary recommendation</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="41" t="str">
+        <x:v>Reach -25%</x:v>
+      </x:c>
+      <x:c r="B6" s="41" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C6" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D6" s="42" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="E6" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F6" s="42" t="n">
+        <x:f>B6*C6*D6/E6</x:f>
+        <x:v>2.88</x:v>
+      </x:c>
+      <x:c r="G6" s="42" t="n">
+        <x:f>F6*5*5/25</x:f>
+        <x:v>2.88</x:v>
+      </x:c>
+      <x:c r="H6" s="41" t="str">
+        <x:v>Tests whether smaller addressable volume changes the decision</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="41" t="str">
+        <x:v>Impact -1</x:v>
+      </x:c>
+      <x:c r="B7" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C7" s="41" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D7" s="42" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="E7" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F7" s="42" t="n">
+        <x:f>B7*C7*D7/E7</x:f>
+        <x:v>2.56</x:v>
+      </x:c>
+      <x:c r="G7" s="42" t="n">
+        <x:f>F7*5*5/25</x:f>
+        <x:v>2.56</x:v>
+      </x:c>
+      <x:c r="H7" s="41" t="str">
+        <x:v>Tests a meaningful rather than trust-critical impact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="41" t="str">
+        <x:v>Confidence -0.2</x:v>
+      </x:c>
+      <x:c r="B8" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C8" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D8" s="42" t="n">
+        <x:v>0.6</x:v>
+      </x:c>
+      <x:c r="E8" s="41" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F8" s="42" t="n">
+        <x:f>B8*C8*D8/E8</x:f>
+        <x:v>2.88</x:v>
+      </x:c>
+      <x:c r="G8" s="42" t="n">
+        <x:f>F8*5*5/25</x:f>
+        <x:v>2.88</x:v>
+      </x:c>
+      <x:c r="H8" s="41" t="str">
+        <x:v>Reflects weaker public-evidence confidence</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="41" t="str">
+        <x:v>Effort +2</x:v>
+      </x:c>
+      <x:c r="B9" s="41" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="C9" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D9" s="42" t="n">
+        <x:v>0.8</x:v>
+      </x:c>
+      <x:c r="E9" s="41" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="F9" s="42" t="n">
+        <x:f>B9*C9*D9/E9</x:f>
+        <x:v>2.7428571428571433</x:v>
+      </x:c>
+      <x:c r="G9" s="42" t="n">
+        <x:f>F9*5*5/25</x:f>
+        <x:v>2.7428571428571433</x:v>
+      </x:c>
+      <x:c r="H9" s="41" t="str">
+        <x:v>Reflects added integration or operational cost</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="42" customHeight="1">
+      <x:c r="A10" s="41" t="str">
+        <x:v>Refund transparency comparator</x:v>
+      </x:c>
+      <x:c r="B10" s="41" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C10" s="41" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="D10" s="42" t="n">
+        <x:v>0.85</x:v>
+      </x:c>
+      <x:c r="E10" s="41" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="F10" s="42" t="n">
+        <x:f>B10*C10*D10/E10</x:f>
+        <x:v>3.8249999999999997</x:v>
+      </x:c>
+      <x:c r="G10" s="42" t="n">
+        <x:f>F10*5*5/25</x:f>
+        <x:v>3.825</x:v>
+      </x:c>
+      <x:c r="H10" s="41" t="str">
+        <x:v>Adjacent option for comparison; not the selected MVP</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>